<commit_message>
Feat: precargar resultados de Catar 1-1 Suiza y Brasil 1-1 Marruecos y actualizar Excel
</commit_message>
<xml_diff>
--- a/Mundial 2026 - Reporte Maestro de Simulaciones.xlsx
+++ b/Mundial 2026 - Reporte Maestro de Simulaciones.xlsx
@@ -787,7 +787,7 @@
       </c>
       <c r="K6" s="5" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>E</t>
         </is>
       </c>
       <c r="L6" s="3" t="n">
@@ -837,7 +837,7 @@
       </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
-          <t>L</t>
+          <t>E</t>
         </is>
       </c>
       <c r="L7" s="3" t="n">

</xml_diff>